<commit_message>
updated agency urls based on responses from FY24 data call
</commit_message>
<xml_diff>
--- a/bin/agency_urls_source.xlsx
+++ b/bin/agency_urls_source.xlsx
@@ -5,10 +5,10 @@
   <workbookPr/>
   <mc:AlternateContent xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006">
     <mc:Choice Requires="x15">
-      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa-github\bin\"/>
+      <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{D956C054-4EB9-4A2A-9B04-DDBFB98B7B93}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78111932-4726-4540-9D83-634C75C7D57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="123" uniqueCount="123">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
   <si>
     <t xml:space="preserve">                Federal Communications Commission (FCC)</t>
   </si>
@@ -195,9 +195,6 @@
     <t>https://www.fws.gov/program/information-quality</t>
   </si>
   <si>
-    <t>https://www.boem.gov/about-boem/regulations-guidance/information-quality</t>
-  </si>
-  <si>
     <t>https://www.usbr.gov/main/qoi/responses.html</t>
   </si>
   <si>
@@ -216,9 +213,6 @@
     <t>https://www.osmre.gov/laws-and-regulations/information-quality</t>
   </si>
   <si>
-    <t>https://www.aphis.usda.gov/aphis/ourfocus/science/sa_peer_reviews</t>
-  </si>
-  <si>
     <t>https://www.energy.gov/cio/department-energy-information-quality-guidelines</t>
   </si>
   <si>
@@ -321,9 +315,6 @@
     <t>https://www.ssa.gov/515/requests.htm</t>
   </si>
   <si>
-    <t>https://www.usgs.gov/office-of-science-quality-and-integrity/information-quality-usgs-peer-review-agenda</t>
-  </si>
-  <si>
     <t>https://www.fws.gov/library/categories/peer-review-plans</t>
   </si>
   <si>
@@ -360,9 +351,6 @@
     <t xml:space="preserve">                Department of the Interior - Office of Surface Mining Reclamation and Enforcement (DOI-OSMRE)</t>
   </si>
   <si>
-    <t>https://www.bsee.gov/what-we-do/research/peer-review</t>
-  </si>
-  <si>
     <t>https://www.bsee.gov/what-we-do/research/peer-review/information-quality</t>
   </si>
   <si>
@@ -394,6 +382,84 @@
   </si>
   <si>
     <t xml:space="preserve">                Department of Agriculture - Economic Research Service (USDA-ERS)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Health and Human Services - National Institutes of Health (HHS-NIH)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Health and Human Services - Food and Drug Administration (HHS-FDA)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Health and Human Services - Centers for Disease Control and Prevention (HHS-CDC)</t>
+  </si>
+  <si>
+    <t>https://www.cdc.gov/science-quality/php/information-quality-support/cdc-atsdr-peer-review-agenda.html</t>
+  </si>
+  <si>
+    <t>https://www.fda.gov/science-research/science-and-research-special-topics/peer-review-scientific-information-and-assessments</t>
+  </si>
+  <si>
+    <t>https://dpcpsi.nih.gov/oepr/infoquality</t>
+  </si>
+  <si>
+    <t>https://www.aphis.usda.gov/peer-review</t>
+  </si>
+  <si>
+    <t>https://www.dol.gov/agencies/ebsa/laws-and-regulations/rules-and-regulations/peer-review/ebsas-response-to-peer-review-reports</t>
+  </si>
+  <si>
+    <t>https://www2.ed.gov/policy/gen/guid/iq/peerreview.html</t>
+  </si>
+  <si>
+    <t>Federal Maritime Commission</t>
+  </si>
+  <si>
+    <t>https://www.fmc.gov/about/information-quality-guidelines/#information-quality-bulletin-for-peer-review-disclaimer</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.boem.gov/about-boem/regulations-guidance/information-quality </t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://www.boem.gov/environment/environmental-studies/boem-science-integrity-quality </t>
+  </si>
+  <si>
+    <t>https://www.bsee.gov/peer-review</t>
+  </si>
+  <si>
+    <t>https://www.usgs.gov/office-of-science-quality-and-integrity/fundamental-science-practices/information-quality-usgs-peer-review-agenda</t>
+  </si>
+  <si>
+    <t>https://www.federalreserve.gov/iq_correction.htm</t>
+  </si>
+  <si>
+    <t>Federal Housing Finance Agency</t>
+  </si>
+  <si>
+    <t>https://www.fhfa.gov/about/information-quality</t>
+  </si>
+  <si>
+    <t>https://www.ed.gov/about/ed-overview/required-notices/information-quality-guidelines/information-correction-requests-and-appeals--information-quality-guidelines</t>
+  </si>
+  <si>
+    <t>National Archives and Records Administration</t>
+  </si>
+  <si>
+    <t>https://www.archives.gov/about/info-qual/requests</t>
+  </si>
+  <si>
+    <t>https://www.fmc.gov/about/information-quality-guidelines/</t>
+  </si>
+  <si>
+    <t>https://www.ntsb.gov/about/Policies/Pages/quality.aspx</t>
+  </si>
+  <si>
+    <t>National Transportation Safety Board (NTSB)</t>
+  </si>
+  <si>
+    <t>https://www.dnfsb.gov/documents</t>
+  </si>
+  <si>
+    <t>Defense Nuclear Facilities Safety Board (DNFSB)</t>
   </si>
 </sst>
 </file>
@@ -725,7 +791,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D49"/>
+  <dimension ref="A1:D57"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="99.85546875" style="1" customWidth="1"/>
@@ -736,24 +802,27 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>120</v>
+        <v>116</v>
       </c>
       <c r="B1" t="s">
-        <v>114</v>
+        <v>110</v>
       </c>
       <c r="C1" t="s">
-        <v>115</v>
+        <v>111</v>
       </c>
       <c r="D1" t="s">
-        <v>116</v>
+        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A2" s="1" t="s">
         <v>1</v>
       </c>
-      <c r="B2" t="s">
+      <c r="B2" s="2" t="s">
         <v>19</v>
+      </c>
+      <c r="C2" s="2" t="s">
+        <v>134</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -766,13 +835,13 @@
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>67</v>
+        <v>65</v>
       </c>
       <c r="B4" s="2" t="s">
         <v>21</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>101</v>
+        <v>98</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -785,7 +854,7 @@
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>68</v>
+        <v>66</v>
       </c>
       <c r="B6" t="s">
         <v>23</v>
@@ -796,7 +865,7 @@
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="B7" t="s">
         <v>25</v>
@@ -818,23 +887,23 @@
         <v>27</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>122</v>
+        <v>118</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>121</v>
+        <v>117</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>69</v>
+        <v>67</v>
       </c>
       <c r="B11" t="s">
         <v>28</v>
@@ -843,13 +912,13 @@
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>84</v>
+        <v>82</v>
       </c>
       <c r="B12" t="s">
         <v>29</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>80</v>
+        <v>78</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -862,7 +931,7 @@
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>70</v>
+        <v>68</v>
       </c>
       <c r="B14" t="s">
         <v>31</v>
@@ -876,12 +945,12 @@
         <v>32</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>102</v>
+        <v>99</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>71</v>
+        <v>69</v>
       </c>
       <c r="B16" t="s">
         <v>34</v>
@@ -897,7 +966,7 @@
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>72</v>
+        <v>70</v>
       </c>
       <c r="B18" t="s">
         <v>36</v>
@@ -905,7 +974,7 @@
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>73</v>
+        <v>71</v>
       </c>
       <c r="B19" t="s">
         <v>37</v>
@@ -916,7 +985,13 @@
         <v>10</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>66</v>
+        <v>64</v>
+      </c>
+      <c r="C20" t="s">
+        <v>127</v>
+      </c>
+      <c r="D20" s="2" t="s">
+        <v>137</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -935,7 +1010,7 @@
         <v>40</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -946,298 +1021,387 @@
         <v>41</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>118</v>
+        <v>114</v>
       </c>
       <c r="B24" t="s">
         <v>42</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="B25" t="s">
-        <v>43</v>
-      </c>
+        <v>121</v>
+      </c>
+      <c r="B25" s="2" t="s">
+        <v>122</v>
+      </c>
+      <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="B26" t="s">
-        <v>44</v>
-      </c>
-      <c r="C26" t="s">
-        <v>45</v>
-      </c>
+        <v>120</v>
+      </c>
+      <c r="B26" s="2" t="s">
+        <v>123</v>
+      </c>
+      <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>117</v>
-      </c>
-      <c r="B27" t="s">
-        <v>46</v>
-      </c>
-      <c r="C27" s="2" t="s">
-        <v>94</v>
-      </c>
+        <v>119</v>
+      </c>
+      <c r="B27" s="2" t="s">
+        <v>124</v>
+      </c>
+      <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>14</v>
+        <v>72</v>
       </c>
       <c r="B28" t="s">
-        <v>47</v>
-      </c>
-      <c r="C28" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>76</v>
+        <v>84</v>
       </c>
       <c r="B29" t="s">
-        <v>49</v>
+        <v>44</v>
+      </c>
+      <c r="C29" t="s">
+        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>75</v>
+        <v>113</v>
       </c>
       <c r="B30" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>97</v>
+        <v>92</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>91</v>
+        <v>14</v>
       </c>
       <c r="B31" t="s">
-        <v>52</v>
-      </c>
-      <c r="C31" s="2" t="s">
-        <v>103</v>
-      </c>
-      <c r="D31" s="2" t="s">
-        <v>106</v>
+        <v>47</v>
+      </c>
+      <c r="C31" t="s">
+        <v>48</v>
       </c>
     </row>
     <row r="32" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A32" s="1" t="s">
-        <v>15</v>
+        <v>74</v>
       </c>
       <c r="B32" t="s">
-        <v>53</v>
+        <v>49</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>88</v>
-      </c>
-      <c r="B33" s="2" t="s">
-        <v>50</v>
+        <v>73</v>
+      </c>
+      <c r="B33" t="s">
+        <v>51</v>
       </c>
       <c r="C33" s="2" t="s">
-        <v>33</v>
-      </c>
-      <c r="D33" s="2" t="s">
-        <v>79</v>
+        <v>95</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>78</v>
+        <v>89</v>
       </c>
       <c r="B34" t="s">
-        <v>54</v>
+        <v>52</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>98</v>
+        <v>100</v>
+      </c>
+      <c r="D34" s="2" t="s">
+        <v>103</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>77</v>
+        <v>15</v>
       </c>
       <c r="B35" t="s">
-        <v>55</v>
-      </c>
-      <c r="C35" s="2" t="s">
-        <v>99</v>
+        <v>53</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A36" s="1" t="s">
-        <v>82</v>
-      </c>
-      <c r="B36" t="s">
-        <v>56</v>
+        <v>86</v>
+      </c>
+      <c r="B36" s="2" t="s">
+        <v>50</v>
       </c>
       <c r="C36" s="2" t="s">
-        <v>100</v>
+        <v>33</v>
+      </c>
+      <c r="D36" s="2" t="s">
+        <v>77</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>89</v>
+        <v>76</v>
       </c>
       <c r="B37" t="s">
-        <v>57</v>
+        <v>54</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>104</v>
+        <v>133</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="B38" s="2" t="s">
-        <v>107</v>
-      </c>
-      <c r="C38" s="2"/>
+        <v>75</v>
+      </c>
+      <c r="B38" t="s">
+        <v>55</v>
+      </c>
+      <c r="C38" s="2" t="s">
+        <v>96</v>
+      </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>108</v>
+        <v>80</v>
       </c>
       <c r="B39" s="2" t="s">
-        <v>58</v>
-      </c>
-      <c r="C39" s="2"/>
+        <v>130</v>
+      </c>
+      <c r="C39" s="2" t="s">
+        <v>97</v>
+      </c>
+      <c r="D39" s="2" t="s">
+        <v>131</v>
+      </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>83</v>
-      </c>
-      <c r="B40" s="2" t="s">
-        <v>59</v>
+        <v>87</v>
+      </c>
+      <c r="B40" t="s">
+        <v>56</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>101</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>16</v>
-      </c>
-      <c r="B41" t="s">
-        <v>60</v>
-      </c>
+        <v>79</v>
+      </c>
+      <c r="B41" s="2" t="s">
+        <v>104</v>
+      </c>
+      <c r="C41" s="2"/>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="B42" t="s">
-        <v>61</v>
+        <v>105</v>
+      </c>
+      <c r="B42" s="2" t="s">
+        <v>57</v>
+      </c>
+      <c r="C42" s="2" t="s">
+        <v>126</v>
       </c>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="B43" t="s">
-        <v>38</v>
+        <v>81</v>
+      </c>
+      <c r="B43" s="2" t="s">
+        <v>58</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>110</v>
+        <v>16</v>
       </c>
       <c r="B44" t="s">
-        <v>62</v>
+        <v>59</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A45" s="1" t="s">
-        <v>17</v>
-      </c>
-      <c r="B45" s="2" t="s">
-        <v>63</v>
-      </c>
-      <c r="C45" s="2" t="s">
-        <v>109</v>
+        <v>115</v>
+      </c>
+      <c r="B45" t="s">
+        <v>60</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>18</v>
+        <v>9</v>
       </c>
       <c r="B46" t="s">
-        <v>64</v>
+        <v>38</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A47" s="1" t="s">
-        <v>0</v>
+        <v>107</v>
       </c>
       <c r="B47" t="s">
-        <v>65</v>
-      </c>
-      <c r="C47" s="2" t="s">
-        <v>105</v>
+        <v>61</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="B48" t="s">
-        <v>96</v>
+        <v>17</v>
+      </c>
+      <c r="B48" s="2" t="s">
+        <v>125</v>
+      </c>
+      <c r="C48" s="2" t="s">
+        <v>106</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A49" s="1" t="s">
-        <v>113</v>
+        <v>18</v>
       </c>
       <c r="B49" t="s">
-        <v>111</v>
-      </c>
-      <c r="C49" s="2" t="s">
-        <v>112</v>
+        <v>62</v>
+      </c>
+    </row>
+    <row r="50" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A50" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="B50" t="s">
+        <v>63</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>102</v>
+      </c>
+    </row>
+    <row r="51" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A51" s="1" t="s">
+        <v>93</v>
+      </c>
+      <c r="B51" t="s">
+        <v>94</v>
+      </c>
+    </row>
+    <row r="52" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A52" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="B52" s="2" t="s">
+        <v>132</v>
+      </c>
+      <c r="C52" s="2" t="s">
+        <v>108</v>
+      </c>
+    </row>
+    <row r="53" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A53" s="1" t="s">
+        <v>128</v>
+      </c>
+      <c r="B53" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C53" s="2" t="s">
+        <v>140</v>
+      </c>
+    </row>
+    <row r="54" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A54" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="B54" s="2" t="s">
+        <v>136</v>
+      </c>
+    </row>
+    <row r="55" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A55" s="1" t="s">
+        <v>138</v>
+      </c>
+      <c r="B55" s="2" t="s">
+        <v>139</v>
+      </c>
+    </row>
+    <row r="56" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A56" s="1" t="s">
+        <v>142</v>
+      </c>
+      <c r="B56" t="s">
+        <v>141</v>
+      </c>
+    </row>
+    <row r="57" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A57" s="1" t="s">
+        <v>144</v>
+      </c>
+      <c r="B57" s="2" t="s">
+        <v>143</v>
       </c>
     </row>
   </sheetData>
   <hyperlinks>
     <hyperlink ref="B20" r:id="rId1" xr:uid="{E9ACD3D3-7C99-4E40-A47C-D00A5EAC955B}"/>
-    <hyperlink ref="B33" r:id="rId2" xr:uid="{25AA9D33-56D6-4FF7-9ACB-387B74AE066D}"/>
-    <hyperlink ref="C33" r:id="rId3" xr:uid="{412C098D-5D66-46B4-B2C9-7A56A185E1E4}"/>
-    <hyperlink ref="D33" r:id="rId4" xr:uid="{2F387A7C-DA92-48B9-AC2A-EBE23A714859}"/>
+    <hyperlink ref="B36" r:id="rId2" xr:uid="{25AA9D33-56D6-4FF7-9ACB-387B74AE066D}"/>
+    <hyperlink ref="C36" r:id="rId3" xr:uid="{412C098D-5D66-46B4-B2C9-7A56A185E1E4}"/>
+    <hyperlink ref="D36" r:id="rId4" xr:uid="{2F387A7C-DA92-48B9-AC2A-EBE23A714859}"/>
     <hyperlink ref="B4" r:id="rId5" xr:uid="{B999D09F-34B3-4977-900A-0E174967434B}"/>
     <hyperlink ref="C23" r:id="rId6" xr:uid="{E83AC65A-CA7E-4D02-B33A-2F8B27D910EB}"/>
     <hyperlink ref="C9" r:id="rId7" xr:uid="{176CC5A5-7F1E-4DD6-A482-7FC0F5EBFE72}"/>
     <hyperlink ref="C22" r:id="rId8" xr:uid="{B8F5DB1F-29A7-4DA4-8823-14EFEBFCE67C}"/>
     <hyperlink ref="C24" r:id="rId9" xr:uid="{C0CCF9F6-332D-4FE4-A994-B3FDA6932409}"/>
-    <hyperlink ref="C27" r:id="rId10" xr:uid="{00C6021A-0390-439A-8E51-956A48392B7B}"/>
-    <hyperlink ref="C30" r:id="rId11" xr:uid="{09C911C3-6D7A-4179-A236-FC1087BABF29}"/>
-    <hyperlink ref="C34" r:id="rId12" xr:uid="{7F2479E3-589B-48B3-84C4-5EE3B3968EE7}"/>
-    <hyperlink ref="C35" r:id="rId13" xr:uid="{A963838C-7062-4271-91E9-7CBA0264B717}"/>
-    <hyperlink ref="C36" r:id="rId14" xr:uid="{A5E328BD-65AA-4AF4-8FA0-80285673B40F}"/>
-    <hyperlink ref="C4" r:id="rId15" xr:uid="{11824155-371F-485B-8804-6F1C29DC62B5}"/>
-    <hyperlink ref="C12" r:id="rId16" xr:uid="{9A1FA534-214D-4FD8-A998-880C44FBE22C}"/>
-    <hyperlink ref="C15" r:id="rId17" xr:uid="{B7B400A6-B288-4CE3-9DCC-C4F07A31D652}"/>
-    <hyperlink ref="C31" r:id="rId18" xr:uid="{A4189098-8366-47CF-BA16-7EBE33B658CA}"/>
-    <hyperlink ref="C37" r:id="rId19" xr:uid="{5111072E-EB5D-4161-9111-01179355DA8F}"/>
-    <hyperlink ref="C47" r:id="rId20" xr:uid="{7FD4C318-1324-4FCE-841F-1E28E6342673}"/>
-    <hyperlink ref="D31" r:id="rId21" xr:uid="{340BE8AF-4D3E-4630-8E09-58D68FC15FE3}"/>
-    <hyperlink ref="B39" r:id="rId22" xr:uid="{8298C29E-D14A-440E-9D97-006455FE4BEE}"/>
-    <hyperlink ref="B38" r:id="rId23" xr:uid="{2A8A081D-4189-405A-AF93-8DFA2B0681E7}"/>
-    <hyperlink ref="B40" r:id="rId24" xr:uid="{81C44319-0F83-4734-984F-2EDF14AAA3D1}"/>
-    <hyperlink ref="B45" r:id="rId25" xr:uid="{8571A975-131E-497B-B0BB-BCDD0D92AFBD}"/>
-    <hyperlink ref="C45" r:id="rId26" xr:uid="{568347C0-4959-4DA9-B57D-EDEAF48149B8}"/>
-    <hyperlink ref="C49" r:id="rId27" xr:uid="{9A8BF28B-AA04-4218-B4E3-064A6FB8AA95}"/>
-    <hyperlink ref="B9" r:id="rId28" xr:uid="{FE4D74C6-342C-4D0B-9A33-D05783073FBF}"/>
-    <hyperlink ref="B10" r:id="rId29" xr:uid="{858B4CAD-F690-4B50-8E6A-C840054A0498}"/>
+    <hyperlink ref="C30" r:id="rId10" xr:uid="{00C6021A-0390-439A-8E51-956A48392B7B}"/>
+    <hyperlink ref="C33" r:id="rId11" xr:uid="{09C911C3-6D7A-4179-A236-FC1087BABF29}"/>
+    <hyperlink ref="C38" r:id="rId12" xr:uid="{A963838C-7062-4271-91E9-7CBA0264B717}"/>
+    <hyperlink ref="C39" r:id="rId13" xr:uid="{A5E328BD-65AA-4AF4-8FA0-80285673B40F}"/>
+    <hyperlink ref="C4" r:id="rId14" xr:uid="{11824155-371F-485B-8804-6F1C29DC62B5}"/>
+    <hyperlink ref="C12" r:id="rId15" xr:uid="{9A1FA534-214D-4FD8-A998-880C44FBE22C}"/>
+    <hyperlink ref="C15" r:id="rId16" xr:uid="{B7B400A6-B288-4CE3-9DCC-C4F07A31D652}"/>
+    <hyperlink ref="C34" r:id="rId17" xr:uid="{A4189098-8366-47CF-BA16-7EBE33B658CA}"/>
+    <hyperlink ref="C40" r:id="rId18" xr:uid="{5111072E-EB5D-4161-9111-01179355DA8F}"/>
+    <hyperlink ref="C50" r:id="rId19" xr:uid="{7FD4C318-1324-4FCE-841F-1E28E6342673}"/>
+    <hyperlink ref="D34" r:id="rId20" xr:uid="{340BE8AF-4D3E-4630-8E09-58D68FC15FE3}"/>
+    <hyperlink ref="B42" r:id="rId21" xr:uid="{8298C29E-D14A-440E-9D97-006455FE4BEE}"/>
+    <hyperlink ref="B41" r:id="rId22" xr:uid="{2A8A081D-4189-405A-AF93-8DFA2B0681E7}"/>
+    <hyperlink ref="B43" r:id="rId23" xr:uid="{81C44319-0F83-4734-984F-2EDF14AAA3D1}"/>
+    <hyperlink ref="C48" r:id="rId24" xr:uid="{568347C0-4959-4DA9-B57D-EDEAF48149B8}"/>
+    <hyperlink ref="C52" r:id="rId25" xr:uid="{9A8BF28B-AA04-4218-B4E3-064A6FB8AA95}"/>
+    <hyperlink ref="B9" r:id="rId26" xr:uid="{FE4D74C6-342C-4D0B-9A33-D05783073FBF}"/>
+    <hyperlink ref="B10" r:id="rId27" xr:uid="{858B4CAD-F690-4B50-8E6A-C840054A0498}"/>
+    <hyperlink ref="B25" r:id="rId28" xr:uid="{5DAAC1C4-A1D2-4B4D-8F04-FB9ADDC430C9}"/>
+    <hyperlink ref="B26" r:id="rId29" xr:uid="{7E197A13-D3AC-4AC7-95DB-9039BE9424A1}"/>
+    <hyperlink ref="B27" r:id="rId30" xr:uid="{A0B5C1F2-EE4A-4D17-AE89-B82AA5A308A0}"/>
+    <hyperlink ref="C42" r:id="rId31" xr:uid="{DF3FAEB0-4E91-4D9A-8EFC-0E795BB2EAC3}"/>
+    <hyperlink ref="B53" r:id="rId32" location="information-quality-bulletin-for-peer-review-disclaimer" xr:uid="{89ABEF6A-97DA-44DC-88FD-F10C47D0DF65}"/>
+    <hyperlink ref="B39" r:id="rId33" xr:uid="{1493D25C-89D7-4020-A587-B14058728042}"/>
+    <hyperlink ref="D39" r:id="rId34" xr:uid="{91D4F156-82ED-41ED-96C2-FEDDF044354B}"/>
+    <hyperlink ref="B52" r:id="rId35" xr:uid="{F65A01BD-A71E-403E-B487-7A7D8627550B}"/>
+    <hyperlink ref="C37" r:id="rId36" xr:uid="{0547C741-B5DF-4844-AD4F-CBE784537F20}"/>
+    <hyperlink ref="C2" r:id="rId37" xr:uid="{282C96FB-561E-4124-A2D5-7ADB2DE1E58B}"/>
+    <hyperlink ref="B2" r:id="rId38" xr:uid="{3AD21894-4644-4247-89A5-6EDD10B020BB}"/>
+    <hyperlink ref="B54" r:id="rId39" xr:uid="{20AF70BF-29F9-41D5-B0B2-D33E6CA1DB08}"/>
+    <hyperlink ref="D20" r:id="rId40" xr:uid="{3CCAC256-5795-4BC2-9800-94091D02983C}"/>
+    <hyperlink ref="B55" r:id="rId41" xr:uid="{02DAEFB8-821F-418B-BA8E-ADC3DB1F3BF4}"/>
+    <hyperlink ref="C53" r:id="rId42" xr:uid="{0810B3C3-C3DB-4044-8705-AB5EBDD4551B}"/>
+    <hyperlink ref="B57" r:id="rId43" xr:uid="{55D069F3-6B19-40F2-8AAC-DE2DAC402D90}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added USGS IQA URL
</commit_message>
<xml_diff>
--- a/bin/agency_urls_source.xlsx
+++ b/bin/agency_urls_source.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{78111932-4726-4540-9D83-634C75C7D57C}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{17982417-BE40-456A-A57D-FB2921DC4890}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15840" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -25,7 +25,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="145" uniqueCount="145">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="146" uniqueCount="146">
   <si>
     <t xml:space="preserve">                Federal Communications Commission (FCC)</t>
   </si>
@@ -460,6 +460,9 @@
   </si>
   <si>
     <t>Defense Nuclear Facilities Safety Board (DNFSB)</t>
+  </si>
+  <si>
+    <t>https://www.usgs.gov/office-of-science-quality-and-integrity/fundamental-science-practices/usgs-information-quality-guidelines</t>
   </si>
 </sst>
 </file>
@@ -1168,6 +1171,9 @@
       <c r="C37" s="2" t="s">
         <v>133</v>
       </c>
+      <c r="D37" s="2" t="s">
+        <v>145</v>
+      </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
@@ -1402,6 +1408,7 @@
     <hyperlink ref="B55" r:id="rId41" xr:uid="{02DAEFB8-821F-418B-BA8E-ADC3DB1F3BF4}"/>
     <hyperlink ref="C53" r:id="rId42" xr:uid="{0810B3C3-C3DB-4044-8705-AB5EBDD4551B}"/>
     <hyperlink ref="B57" r:id="rId43" xr:uid="{55D069F3-6B19-40F2-8AAC-DE2DAC402D90}"/>
+    <hyperlink ref="D37" r:id="rId44" xr:uid="{DDD7C9ED-C6F0-4136-8986-6B3653FDE430}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
Updated URL list to include new links for Census and DOE/DOE labs.  Deleted empty whitespace and typos in peer review source file which were returing warnings and artifacts in .csv files for FY11 and FY16
</commit_message>
<xml_diff>
--- a/bin/agency_urls_source.xlsx
+++ b/bin/agency_urls_source.xlsx
@@ -8,9 +8,9 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{3DFB37BE-5951-4BC7-AEBD-7CDC35A08BF5}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{91D2DE61-733E-4143-88F5-580947150E98}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="1950" yWindow="1215" windowWidth="27510" windowHeight="13320" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
@@ -20,12 +20,15 @@
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
     </ext>
+    <ext xmlns:xlwcv="http://schemas.microsoft.com/office/spreadsheetml/2024/workbookCompatibilityVersion" uri="{D14903EA-33C4-47F7-8F05-3474C54BE107}">
+      <xlwcv:version setVersion="1"/>
+    </ext>
   </extLst>
 </workbook>
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="148" uniqueCount="148">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="153" uniqueCount="153">
   <si>
     <t xml:space="preserve">                Federal Communications Commission (FCC)</t>
   </si>
@@ -81,9 +84,6 @@
     <t xml:space="preserve">                Department of Agriculture - Animal and Plant Health Inspection Service (USDA-APHIS)</t>
   </si>
   <si>
-    <t xml:space="preserve">                Department of Energy (DOE)</t>
-  </si>
-  <si>
     <t>https://www.federalreserve.gov/iq_guidelines.htm</t>
   </si>
   <si>
@@ -469,6 +469,24 @@
   </si>
   <si>
     <t xml:space="preserve">                Department of Commerce - National Institute of Standards &amp; Technology (DOC-NIST)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Department of Energy (DOE) - Department-wide resources</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Department of Energy (DOE) - National Energy Technology Laboratory (DOE-NETL)</t>
+  </si>
+  <si>
+    <t xml:space="preserve">https://netl.doe.gov/peerreviews </t>
+  </si>
+  <si>
+    <t>https://www.directives.doe.gov/terms_definitions/peer-review-1</t>
+  </si>
+  <si>
+    <t>https://www.census.gov/quality/</t>
+  </si>
+  <si>
+    <t xml:space="preserve">                Department of Commerce - U.S. Census Bureau (DOC-Census)</t>
   </si>
 </sst>
 </file>
@@ -800,7 +818,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D58"/>
+  <dimension ref="A1:D60"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="99.85546875" style="1" customWidth="1"/>
@@ -811,16 +829,16 @@
   <sheetData>
     <row r="1" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A1" s="1" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="B1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C1" t="s">
         <v>110</v>
       </c>
-      <c r="C1" t="s">
+      <c r="D1" t="s">
         <v>111</v>
-      </c>
-      <c r="D1" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="2" spans="1:4" x14ac:dyDescent="0.25">
@@ -828,10 +846,10 @@
         <v>1</v>
       </c>
       <c r="B2" s="2" t="s">
-        <v>19</v>
+        <v>18</v>
       </c>
       <c r="C2" s="2" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="3" spans="1:4" x14ac:dyDescent="0.25">
@@ -839,18 +857,18 @@
         <v>2</v>
       </c>
       <c r="B3" t="s">
-        <v>20</v>
+        <v>19</v>
       </c>
     </row>
     <row r="4" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A4" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="B4" s="2" t="s">
-        <v>21</v>
+        <v>20</v>
       </c>
       <c r="C4" s="2" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
     </row>
     <row r="5" spans="1:4" x14ac:dyDescent="0.25">
@@ -858,26 +876,26 @@
         <v>3</v>
       </c>
       <c r="B5" t="s">
-        <v>22</v>
+        <v>21</v>
       </c>
     </row>
     <row r="6" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A6" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="B6" t="s">
+        <v>22</v>
+      </c>
+      <c r="C6" t="s">
         <v>23</v>
-      </c>
-      <c r="C6" t="s">
-        <v>24</v>
       </c>
     </row>
     <row r="7" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A7" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="B7" t="s">
-        <v>25</v>
+        <v>24</v>
       </c>
     </row>
     <row r="8" spans="1:4" x14ac:dyDescent="0.25">
@@ -885,7 +903,7 @@
         <v>4</v>
       </c>
       <c r="B8" t="s">
-        <v>26</v>
+        <v>25</v>
       </c>
     </row>
     <row r="9" spans="1:4" x14ac:dyDescent="0.25">
@@ -893,41 +911,41 @@
         <v>5</v>
       </c>
       <c r="B9" s="2" t="s">
-        <v>27</v>
+        <v>26</v>
       </c>
       <c r="C9" s="2" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="D9" s="2"/>
     </row>
     <row r="10" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A10" s="1" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="B10" s="2" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="C10" s="2"/>
       <c r="D10" s="2"/>
     </row>
     <row r="11" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A11" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="B11" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C11" s="2"/>
     </row>
     <row r="12" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A12" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="B12" t="s">
-        <v>29</v>
+        <v>28</v>
       </c>
       <c r="C12" s="2" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
     </row>
     <row r="13" spans="1:4" x14ac:dyDescent="0.25">
@@ -935,15 +953,15 @@
         <v>6</v>
       </c>
       <c r="B13" t="s">
-        <v>30</v>
+        <v>29</v>
       </c>
     </row>
     <row r="14" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A14" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="B14" t="s">
-        <v>31</v>
+        <v>30</v>
       </c>
     </row>
     <row r="15" spans="1:4" x14ac:dyDescent="0.25">
@@ -951,18 +969,18 @@
         <v>7</v>
       </c>
       <c r="B15" t="s">
-        <v>32</v>
+        <v>31</v>
       </c>
       <c r="C15" s="2" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
     </row>
     <row r="16" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A16" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="B16" t="s">
-        <v>34</v>
+        <v>33</v>
       </c>
     </row>
     <row r="17" spans="1:4" x14ac:dyDescent="0.25">
@@ -970,23 +988,23 @@
         <v>8</v>
       </c>
       <c r="B17" t="s">
-        <v>35</v>
+        <v>34</v>
       </c>
     </row>
     <row r="18" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A18" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="B18" t="s">
-        <v>36</v>
+        <v>35</v>
       </c>
     </row>
     <row r="19" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A19" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="B19" t="s">
-        <v>37</v>
+        <v>36</v>
       </c>
     </row>
     <row r="20" spans="1:4" x14ac:dyDescent="0.25">
@@ -994,13 +1012,13 @@
         <v>10</v>
       </c>
       <c r="B20" s="2" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C20" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
       <c r="D20" s="2" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="21" spans="1:4" x14ac:dyDescent="0.25">
@@ -1008,7 +1026,7 @@
         <v>11</v>
       </c>
       <c r="B21" t="s">
-        <v>39</v>
+        <v>38</v>
       </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
@@ -1016,10 +1034,10 @@
         <v>12</v>
       </c>
       <c r="B22" t="s">
-        <v>40</v>
+        <v>39</v>
       </c>
       <c r="C22" s="2" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
     </row>
     <row r="23" spans="1:4" x14ac:dyDescent="0.25">
@@ -1027,86 +1045,86 @@
         <v>13</v>
       </c>
       <c r="B23" t="s">
-        <v>41</v>
+        <v>40</v>
       </c>
       <c r="C23" s="2" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
     </row>
     <row r="24" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A24" s="1" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="B24" t="s">
-        <v>42</v>
+        <v>41</v>
       </c>
       <c r="C24" s="2" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
     </row>
     <row r="25" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A25" s="1" t="s">
+        <v>120</v>
+      </c>
+      <c r="B25" s="2" t="s">
         <v>121</v>
-      </c>
-      <c r="B25" s="2" t="s">
-        <v>122</v>
       </c>
       <c r="C25" s="2"/>
     </row>
     <row r="26" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A26" s="1" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="B26" s="2" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="C26" s="2"/>
     </row>
     <row r="27" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A27" s="1" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="B27" s="2" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="C27" s="2"/>
     </row>
     <row r="28" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A28" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="B28" t="s">
-        <v>43</v>
+        <v>42</v>
       </c>
     </row>
     <row r="29" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A29" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="B29" t="s">
+        <v>43</v>
+      </c>
+      <c r="C29" t="s">
         <v>44</v>
-      </c>
-      <c r="C29" t="s">
-        <v>45</v>
       </c>
     </row>
     <row r="30" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A30" s="1" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="B30" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C30" s="2" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
     </row>
     <row r="31" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A31" s="1" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="B31" s="2" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="C31" s="2"/>
     </row>
@@ -1115,43 +1133,43 @@
         <v>14</v>
       </c>
       <c r="B32" t="s">
+        <v>46</v>
+      </c>
+      <c r="C32" t="s">
         <v>47</v>
-      </c>
-      <c r="C32" t="s">
-        <v>48</v>
       </c>
     </row>
     <row r="33" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A33" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="B33" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
     </row>
     <row r="34" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A34" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="B34" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C34" s="2" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
     </row>
     <row r="35" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A35" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="B35" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C35" s="2" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="D35" s="2" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
     </row>
     <row r="36" spans="1:4" x14ac:dyDescent="0.25">
@@ -1159,99 +1177,99 @@
         <v>15</v>
       </c>
       <c r="B36" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
     </row>
     <row r="37" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A37" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="B37" s="2" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C37" s="2" t="s">
-        <v>33</v>
+        <v>32</v>
       </c>
       <c r="D37" s="2" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
     </row>
     <row r="38" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A38" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="B38" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C38" s="2" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D38" s="2" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="39" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A39" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="B39" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C39" s="2" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
     </row>
     <row r="40" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A40" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="B40" s="2" t="s">
+        <v>129</v>
+      </c>
+      <c r="C40" s="2" t="s">
+        <v>96</v>
+      </c>
+      <c r="D40" s="2" t="s">
         <v>130</v>
-      </c>
-      <c r="C40" s="2" t="s">
-        <v>97</v>
-      </c>
-      <c r="D40" s="2" t="s">
-        <v>131</v>
       </c>
     </row>
     <row r="41" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A41" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="B41" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C41" s="2" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
     </row>
     <row r="42" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A42" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="B42" s="2" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C42" s="2"/>
     </row>
     <row r="43" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A43" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="B43" s="2" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C43" s="2" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="44" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A44" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="B44" s="2" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
     </row>
     <row r="45" spans="1:4" x14ac:dyDescent="0.25">
@@ -1259,15 +1277,15 @@
         <v>16</v>
       </c>
       <c r="B45" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
     </row>
     <row r="46" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A46" s="1" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="B46" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
     </row>
     <row r="47" spans="1:4" x14ac:dyDescent="0.25">
@@ -1275,15 +1293,15 @@
         <v>9</v>
       </c>
       <c r="B47" t="s">
-        <v>38</v>
+        <v>37</v>
       </c>
     </row>
     <row r="48" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A48" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="B48" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
     </row>
     <row r="49" spans="1:3" x14ac:dyDescent="0.25">
@@ -1291,18 +1309,21 @@
         <v>17</v>
       </c>
       <c r="B49" s="2" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="C49" s="2" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
     </row>
     <row r="50" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A50" s="1" t="s">
-        <v>18</v>
+        <v>147</v>
       </c>
       <c r="B50" t="s">
-        <v>62</v>
+        <v>61</v>
+      </c>
+      <c r="C50" s="2" t="s">
+        <v>150</v>
       </c>
     </row>
     <row r="51" spans="1:3" x14ac:dyDescent="0.25">
@@ -1310,72 +1331,88 @@
         <v>0</v>
       </c>
       <c r="B51" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C51" s="2" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
     </row>
     <row r="52" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A52" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="B52" t="s">
         <v>93</v>
-      </c>
-      <c r="B52" t="s">
-        <v>94</v>
       </c>
     </row>
     <row r="53" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A53" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="B53" s="2" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="C53" s="2" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
     </row>
     <row r="54" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A54" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="B54" s="2" t="s">
         <v>128</v>
       </c>
-      <c r="B54" s="2" t="s">
-        <v>129</v>
-      </c>
       <c r="C54" s="2" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="55" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A55" s="1" t="s">
+        <v>134</v>
+      </c>
+      <c r="B55" s="2" t="s">
         <v>135</v>
-      </c>
-      <c r="B55" s="2" t="s">
-        <v>136</v>
       </c>
     </row>
     <row r="56" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A56" s="1" t="s">
+        <v>137</v>
+      </c>
+      <c r="B56" s="2" t="s">
         <v>138</v>
-      </c>
-      <c r="B56" s="2" t="s">
-        <v>139</v>
       </c>
     </row>
     <row r="57" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A57" s="1" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="B57" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="58" spans="1:3" x14ac:dyDescent="0.25">
       <c r="A58" s="1" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="B58" s="2" t="s">
-        <v>143</v>
+        <v>142</v>
+      </c>
+    </row>
+    <row r="59" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A59" s="1" t="s">
+        <v>148</v>
+      </c>
+      <c r="B59" s="2" t="s">
+        <v>149</v>
+      </c>
+    </row>
+    <row r="60" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A60" s="1" t="s">
+        <v>152</v>
+      </c>
+      <c r="B60" s="2" t="s">
+        <v>151</v>
       </c>
     </row>
   </sheetData>
@@ -1425,6 +1462,9 @@
     <hyperlink ref="B58" r:id="rId43" xr:uid="{55D069F3-6B19-40F2-8AAC-DE2DAC402D90}"/>
     <hyperlink ref="D38" r:id="rId44" xr:uid="{DDD7C9ED-C6F0-4136-8986-6B3653FDE430}"/>
     <hyperlink ref="B31" r:id="rId45" xr:uid="{045552A8-E80E-4B2C-B7B8-6982276AB0EC}"/>
+    <hyperlink ref="B59" r:id="rId46" xr:uid="{A8B79102-D0CE-404E-BF5E-12F44ED791F3}"/>
+    <hyperlink ref="C50" r:id="rId47" xr:uid="{2723915E-460B-4294-B64C-8D55F1B6649C}"/>
+    <hyperlink ref="B60" r:id="rId48" xr:uid="{DA482807-DB96-4FBA-9BAC-EB39599C6687}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
added FY25 data.  small formatting changes to 'organization type' to fit chart
</commit_message>
<xml_diff>
--- a/bin/agency_urls_source.xlsx
+++ b/bin/agency_urls_source.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="F:\IQA\iqa\bin\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{9CA0A2A7-3624-4AAF-BED8-D0B739085807}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{2F02B0BB-A54D-41A1-93B8-5B27FEC51979}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-120" yWindow="-120" windowWidth="29040" windowHeight="15720" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
@@ -28,7 +28,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="160" uniqueCount="160">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="173" uniqueCount="173">
   <si>
     <t xml:space="preserve">                Federal Communications Commission (FCC)</t>
   </si>
@@ -508,6 +508,45 @@
   </si>
   <si>
     <t xml:space="preserve">                Department of Commerce - Bureau of Industry and Security (DOC-BIS)</t>
+  </si>
+  <si>
+    <t>https://www.ttb.gov/public-information</t>
+  </si>
+  <si>
+    <t>Department of the Treasury - Alcohol and Tobacco Tax and Trade Bureau (TREAS-TTB)</t>
+  </si>
+  <si>
+    <t>https://fiscal.treasury.gov/data-quality/index.html</t>
+  </si>
+  <si>
+    <t>Department of the Treasury - Bureau of the Fiscal Service (TREAS-BFS)</t>
+  </si>
+  <si>
+    <t>https://home.treasury.gov/information-quality-program</t>
+  </si>
+  <si>
+    <t>https://www.fincen.gov/system/files/shared/515procedures2.pdf</t>
+  </si>
+  <si>
+    <t>https://www.irs.gov/pub/newsroom/infoqualityguidelines.pdf</t>
+  </si>
+  <si>
+    <t>Department of the Treasury - Financial Crimes Enforcement Network (TREAS-FINCEN)</t>
+  </si>
+  <si>
+    <t>Department of the Treasury - Internal Revenue Service (TREAS-IRS)</t>
+  </si>
+  <si>
+    <t>https://home.treasury.gov/system/files/236/Information-Quality-Guidelines.pdf</t>
+  </si>
+  <si>
+    <t>Department of the Treasury - Office of Comptroller of the Currency (TREAS-OCC)</t>
+  </si>
+  <si>
+    <t>Department of the Treasury - U.S. Mint (TREAS-MINT)</t>
+  </si>
+  <si>
+    <t>https://www.usmint.gov/resources/information-quality</t>
   </si>
 </sst>
 </file>
@@ -839,7 +878,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{00000000-0001-0000-0000-000000000000}">
-  <dimension ref="A1:D63"/>
+  <dimension ref="A1:D69"/>
   <sheetFormatPr defaultRowHeight="15" x14ac:dyDescent="0.25"/>
   <cols>
     <col min="1" max="1" width="99.85546875" style="1" customWidth="1"/>
@@ -1052,6 +1091,9 @@
       <c r="B21" t="s">
         <v>38</v>
       </c>
+      <c r="C21" s="2" t="s">
+        <v>164</v>
+      </c>
     </row>
     <row r="22" spans="1:4" x14ac:dyDescent="0.25">
       <c r="A22" s="1" t="s">
@@ -1461,6 +1503,55 @@
       </c>
       <c r="B63" t="s">
         <v>158</v>
+      </c>
+    </row>
+    <row r="64" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A64" s="1" t="s">
+        <v>161</v>
+      </c>
+      <c r="B64" t="s">
+        <v>160</v>
+      </c>
+    </row>
+    <row r="65" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A65" s="1" t="s">
+        <v>163</v>
+      </c>
+      <c r="B65" t="s">
+        <v>162</v>
+      </c>
+    </row>
+    <row r="66" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A66" s="1" t="s">
+        <v>167</v>
+      </c>
+      <c r="B66" t="s">
+        <v>165</v>
+      </c>
+    </row>
+    <row r="67" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A67" s="1" t="s">
+        <v>168</v>
+      </c>
+      <c r="B67" t="s">
+        <v>166</v>
+      </c>
+    </row>
+    <row r="68" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A68" s="1" t="s">
+        <v>170</v>
+      </c>
+      <c r="B68" s="2" t="s">
+        <v>169</v>
+      </c>
+      <c r="C68" s="2"/>
+    </row>
+    <row r="69" spans="1:3" x14ac:dyDescent="0.25">
+      <c r="A69" s="1" t="s">
+        <v>171</v>
+      </c>
+      <c r="B69" t="s">
+        <v>172</v>
       </c>
     </row>
   </sheetData>
@@ -1514,6 +1605,8 @@
     <hyperlink ref="C50" r:id="rId47" xr:uid="{2723915E-460B-4294-B64C-8D55F1B6649C}"/>
     <hyperlink ref="B60" r:id="rId48" xr:uid="{DA482807-DB96-4FBA-9BAC-EB39599C6687}"/>
     <hyperlink ref="D15" r:id="rId49" xr:uid="{641233B5-DC48-4B29-BC04-78B4E8ECBF8B}"/>
+    <hyperlink ref="C21" r:id="rId50" xr:uid="{43C88833-BE37-45CA-8822-080320873161}"/>
+    <hyperlink ref="B68" r:id="rId51" xr:uid="{B08A1D42-9236-4838-B5A3-2694BF0B0540}"/>
   </hyperlinks>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>